<commit_message>
Sync from sheetspeed-website 64895f2
</commit_message>
<xml_diff>
--- a/DataSniper-Starter-alt.xlsx
+++ b/DataSniper-Starter-alt.xlsx
@@ -3,8 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24106"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet name="DataSniper" sheetId="1" r:id="rId1"/>
+    <sheet name="Start here" sheetId="2" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -38,9 +42,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment wrapText="1" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -71,16 +76,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="96" customWidth="1"/>
+    <col min="1" max="1" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DataSniper starter. This workbook opens with the task pane visible. Save it after you snip, and Excel for Mac keeps the pane with the file.</t>
+          <t>DataSniper is ready. This workbook opens with the task pane visible, and Excel for Mac keeps it visible when you save. Export onto the DataSniper sheet so this note stays put.</t>
         </is>
       </c>
     </row>

</xml_diff>